<commit_message>
Ajuste na prioridade do calculo para os não-comissionados
</commit_message>
<xml_diff>
--- a/vendedores.xlsx
+++ b/vendedores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TI\ROBERT\PROJETO COMISSOES\Script\extrator_comissoes_relatorio_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA00BCC0-A31B-4500-99B9-D5BB7B5975C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8E96828-28AB-407A-BA80-3DBA40417EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VENDEDORES" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Alteração no json final, com a inclusão da ajuda de custo individual e total. Remoção dos .txt
</commit_message>
<xml_diff>
--- a/vendedores.xlsx
+++ b/vendedores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TI\ROBERT\PROJETO COMISSOES\Script\extrator_comissoes_relatorio_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8E96828-28AB-407A-BA80-3DBA40417EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E747EC91-4A14-454B-A386-0BE5AB17123D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="BLACKLIST_CLIENTES" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">VENDEDORES!$A$1:$C$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">VENDEDORES!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="55">
   <si>
     <t>Nome</t>
   </si>
@@ -107,12 +107,6 @@
     <t>ROBERTA_SANTOS</t>
   </si>
   <si>
-    <t>RODRIGO_APARECIDO_BERNADINO</t>
-  </si>
-  <si>
-    <t>RODRIGO_FREIRE</t>
-  </si>
-  <si>
     <t>RODRIGO_MIRANDA</t>
   </si>
   <si>
@@ -195,6 +189,12 @@
   </si>
   <si>
     <t>MATEUS_ARAUJO</t>
+  </si>
+  <si>
+    <t>Ajuda de Custo</t>
+  </si>
+  <si>
+    <t>NÃO</t>
   </si>
 </sst>
 </file>
@@ -276,7 +276,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -285,6 +285,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -589,15 +592,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -607,8 +611,11 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -618,19 +625,25 @@
       <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="D3" s="4">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -638,21 +651,27 @@
         <v>4</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="D4" s="4">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="D5" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
@@ -660,10 +679,13 @@
         <v>4</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="D6" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
@@ -671,10 +693,13 @@
         <v>4</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="D7" s="4">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
@@ -682,10 +707,13 @@
         <v>4</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="D8" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -695,8 +723,11 @@
       <c r="C9" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D9" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>11</v>
       </c>
@@ -706,8 +737,11 @@
       <c r="C10" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D10" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -715,10 +749,13 @@
         <v>4</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="D11" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>13</v>
       </c>
@@ -728,8 +765,11 @@
       <c r="C12" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D12" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>14</v>
       </c>
@@ -739,8 +779,11 @@
       <c r="C13" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D13" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>15</v>
       </c>
@@ -750,8 +793,11 @@
       <c r="C14" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D14" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>16</v>
       </c>
@@ -761,8 +807,11 @@
       <c r="C15" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D15" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>17</v>
       </c>
@@ -770,10 +819,13 @@
         <v>4</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="D16" s="4">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>18</v>
       </c>
@@ -783,8 +835,11 @@
       <c r="C17" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D17" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
@@ -792,10 +847,13 @@
         <v>4</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="D18" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -805,8 +863,11 @@
       <c r="C19" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D19" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>21</v>
       </c>
@@ -816,8 +877,11 @@
       <c r="C20" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D20" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>22</v>
       </c>
@@ -827,8 +891,11 @@
       <c r="C21" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D21" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>23</v>
       </c>
@@ -836,10 +903,13 @@
         <v>4</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="D22" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>24</v>
       </c>
@@ -847,10 +917,13 @@
         <v>4</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="D23" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>25</v>
       </c>
@@ -860,8 +933,11 @@
       <c r="C24" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D24" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>26</v>
       </c>
@@ -869,10 +945,13 @@
         <v>4</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="D25" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>27</v>
       </c>
@@ -882,8 +961,11 @@
       <c r="C26" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D26" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>28</v>
       </c>
@@ -893,8 +975,11 @@
       <c r="C27" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D27" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>29</v>
       </c>
@@ -902,10 +987,13 @@
         <v>4</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="D28" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>30</v>
       </c>
@@ -915,8 +1003,11 @@
       <c r="C29" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D29" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>31</v>
       </c>
@@ -926,8 +1017,11 @@
       <c r="C30" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D30" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>32</v>
       </c>
@@ -937,108 +1031,110 @@
       <c r="C31" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D31" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D32" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="C33" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D33" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D34" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D35" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D36" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D37" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>5</v>
+        <v>54</v>
+      </c>
+      <c r="D38" s="4">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C40" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:D1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1058,42 +1154,42 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1111,12 +1207,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
nova variavel controladora se a data é automatica ou manual
</commit_message>
<xml_diff>
--- a/vendedores.xlsx
+++ b/vendedores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TI\ROBERT\PROJETO COMISSOES\Script\extrator_comissoes_relatorio_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E747EC91-4A14-454B-A386-0BE5AB17123D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D40510B5-931B-49B5-824A-550E8EA10DEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="VENDEDORES" sheetId="1" r:id="rId1"/>
     <sheet name="BLACKLIST_VENDEDORES" sheetId="2" r:id="rId2"/>
     <sheet name="BLACKLIST_CLIENTES" sheetId="3" r:id="rId3"/>
+    <sheet name="COORDENADORES" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">VENDEDORES!$A$1:$D$1</definedName>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="64">
   <si>
     <t>Nome</t>
   </si>
@@ -195,13 +196,40 @@
   </si>
   <si>
     <t>NÃO</t>
+  </si>
+  <si>
+    <t>0.35</t>
+  </si>
+  <si>
+    <t>0.1</t>
+  </si>
+  <si>
+    <t>PEDRO HENRIQUE</t>
+  </si>
+  <si>
+    <t>JOÃO VITOR</t>
+  </si>
+  <si>
+    <t>JOÃO PEDRO</t>
+  </si>
+  <si>
+    <t>SERGIO VITAL</t>
+  </si>
+  <si>
+    <t>EUVERALDO OLIVEIRA</t>
+  </si>
+  <si>
+    <t>ANTONIO PAIVA</t>
+  </si>
+  <si>
+    <t>CARLOS_HENRIQUE_AMARO_DA_SILVA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -218,6 +246,12 @@
     <font>
       <sz val="9"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -592,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -654,29 +688,29 @@
         <v>54</v>
       </c>
       <c r="D4" s="4">
-        <v>20000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>54</v>
       </c>
       <c r="D5" s="4">
-        <v>0</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>54</v>
@@ -687,7 +721,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>4</v>
@@ -696,12 +730,12 @@
         <v>54</v>
       </c>
       <c r="D7" s="4">
-        <v>12000</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>4</v>
@@ -710,26 +744,26 @@
         <v>54</v>
       </c>
       <c r="D8" s="4">
-        <v>0</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="D9" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>4</v>
@@ -738,32 +772,32 @@
         <v>5</v>
       </c>
       <c r="D10" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D11" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="D12" s="4">
         <v>3500</v>
@@ -771,7 +805,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>4</v>
@@ -785,7 +819,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>4</v>
@@ -794,12 +828,12 @@
         <v>5</v>
       </c>
       <c r="D14" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>4</v>
@@ -813,55 +847,55 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D16" s="4">
-        <v>20000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="D17" s="4">
-        <v>3500</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D18" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="D19" s="4">
         <v>0</v>
@@ -869,7 +903,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>4</v>
@@ -878,12 +912,12 @@
         <v>5</v>
       </c>
       <c r="D20" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>4</v>
@@ -897,21 +931,21 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D22" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>4</v>
@@ -920,18 +954,18 @@
         <v>54</v>
       </c>
       <c r="D23" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="D24" s="4">
         <v>3500</v>
@@ -939,13 +973,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D25" s="4">
         <v>3500</v>
@@ -953,13 +987,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="D26" s="4">
         <v>3500</v>
@@ -967,7 +1001,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>4</v>
@@ -981,13 +1015,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D28" s="4">
         <v>3500</v>
@@ -995,21 +1029,21 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="D29" s="4">
-        <v>3500</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>4</v>
@@ -1023,7 +1057,7 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>4</v>
@@ -1037,10 +1071,10 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>5</v>
@@ -1051,7 +1085,7 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>34</v>
@@ -1065,7 +1099,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>34</v>
@@ -1079,7 +1113,7 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>34</v>
@@ -1093,7 +1127,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>34</v>
@@ -1107,7 +1141,7 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>34</v>
@@ -1121,27 +1155,42 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D38" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D39" s="4">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -1190,6 +1239,11 @@
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1218,4 +1272,118 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B6EEA29-FD81-4322-870F-7B3DE2DEC8DC}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D2" s="2">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="2">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="2">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="2">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="2">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="2">
+        <v>3500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
remoção das NFs manifestadas a partir do supabase
</commit_message>
<xml_diff>
--- a/vendedores.xlsx
+++ b/vendedores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TI\ROBERT\PROJETO COMISSOES\Script\extrator_comissoes_relatorio_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96F130F7-5364-45BF-A0B7-1C4BF05CA70E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DFAEF9A-044A-4E5B-9D5B-1890EEB31A2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VENDEDORES" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="65">
   <si>
     <t>Nome</t>
   </si>
@@ -231,14 +231,17 @@
     <t>ANTONIO PAIVA</t>
   </si>
   <si>
-    <t>CARLOS_HENRIQUE_AMARO_DA_SILVA</t>
+    <t>CARLOS_HENRIQUE</t>
+  </si>
+  <si>
+    <t>Lucas_Cacciatore</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -261,6 +264,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -319,7 +327,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -331,6 +339,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -635,7 +646,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -953,8 +964,8 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>23</v>
+      <c r="A23" s="5" t="s">
+        <v>64</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>4</v>
@@ -968,7 +979,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>4</v>
@@ -977,18 +988,18 @@
         <v>54</v>
       </c>
       <c r="D24" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="D25" s="4">
         <v>3500</v>
@@ -996,13 +1007,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D26" s="4">
         <v>3500</v>
@@ -1010,13 +1021,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="D27" s="4">
         <v>3500</v>
@@ -1024,7 +1035,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>4</v>
@@ -1038,35 +1049,35 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D29" s="4">
-        <v>12000</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="D30" s="4">
-        <v>3500</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>4</v>
@@ -1080,7 +1091,7 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>4</v>
@@ -1094,10 +1105,10 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>5</v>
@@ -1108,7 +1119,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>34</v>
@@ -1122,7 +1133,7 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>34</v>
@@ -1136,7 +1147,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>34</v>
@@ -1150,7 +1161,7 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>34</v>
@@ -1164,7 +1175,7 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>34</v>
@@ -1178,15 +1189,29 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D39" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D40" s="4">
         <v>0</v>
       </c>
     </row>
@@ -1194,6 +1219,7 @@
   <autoFilter ref="A1:D1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Ajuste na prioridade dos sem comissao, sobre os 2% do simulador ausente
</commit_message>
<xml_diff>
--- a/vendedores.xlsx
+++ b/vendedores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TI\ROBERT\PROJETO COMISSOES\Script\extrator_comissoes_relatorio_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DFAEF9A-044A-4E5B-9D5B-1890EEB31A2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78255892-A9BD-4C2D-8A9A-76564F34B2E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="66">
   <si>
     <t>Nome</t>
   </si>
@@ -234,7 +234,10 @@
     <t>CARLOS_HENRIQUE</t>
   </si>
   <si>
-    <t>Lucas_Cacciatore</t>
+    <t>DIEGO_FERNANDES</t>
+  </si>
+  <si>
+    <t>LUCAS_CACCIATORE</t>
   </si>
 </sst>
 </file>
@@ -755,7 +758,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>4</v>
@@ -764,12 +767,12 @@
         <v>54</v>
       </c>
       <c r="D8" s="4">
-        <v>12000</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>4</v>
@@ -778,26 +781,26 @@
         <v>54</v>
       </c>
       <c r="D9" s="4">
-        <v>0</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>5</v>
+        <v>54</v>
       </c>
       <c r="D10" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>4</v>
@@ -806,21 +809,21 @@
         <v>5</v>
       </c>
       <c r="D11" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D12" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -965,7 +968,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>4</v>
@@ -1225,7 +1228,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -1279,6 +1282,11 @@
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implementação da separação do diretorio Coordenadores por estado: Simuladores copiados conforme o estado(SP/MG), relatorios gerais apenas um espelho (todos pedidos SP+MG)
</commit_message>
<xml_diff>
--- a/vendedores.xlsx
+++ b/vendedores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TI\ROBERT\PROJETO COMISSOES\Script\extrator_comissoes_relatorio_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78255892-A9BD-4C2D-8A9A-76564F34B2E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DCB7B3A-362E-4DC8-8318-77CFDBD5DF8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VENDEDORES" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="68">
   <si>
     <t>Nome</t>
   </si>
@@ -63,181 +63,187 @@
     <t>ANTONIO_PAIVA</t>
   </si>
   <si>
+    <t>DIEGO_JOSE_ARANTES</t>
+  </si>
+  <si>
+    <t>DIEGO_SOUSA_SANTOS</t>
+  </si>
+  <si>
+    <t>EBER_VIEIRA</t>
+  </si>
+  <si>
+    <t>EDCARLOS_SANTOS_DE_SOUZA</t>
+  </si>
+  <si>
+    <t>FLÁVIO_COUTINHO</t>
+  </si>
+  <si>
+    <t>GABRIEL_BARRETO</t>
+  </si>
+  <si>
+    <t>GABRIEL_DE_DEUS_NICOLAU</t>
+  </si>
+  <si>
+    <t>HUGO_FELIPE_DA_MATA</t>
+  </si>
+  <si>
+    <t>ISAQUE_CARVALHO_DO_ESPIRITO_SANTOS</t>
+  </si>
+  <si>
+    <t>JAMES_MADSON_OLIVEIRA_DE_SOUZA</t>
+  </si>
+  <si>
+    <t>JOARES_ALVES</t>
+  </si>
+  <si>
+    <t>JORGE_LUIZ</t>
+  </si>
+  <si>
+    <t>LARISSA_ALMEIDA</t>
+  </si>
+  <si>
+    <t>LEIDIANE_TEIXEIRA_COSTA</t>
+  </si>
+  <si>
+    <t>LEONARDO_APARECIDO_DE_MORAES</t>
+  </si>
+  <si>
+    <t>LEONARDO_PRATES</t>
+  </si>
+  <si>
+    <t>ROBERTA_SANTOS</t>
+  </si>
+  <si>
+    <t>RODRIGO_MIRANDA</t>
+  </si>
+  <si>
+    <t>RODRIGO_BERNARDINO</t>
+  </si>
+  <si>
+    <t>SARALIGIA_SIMÕES</t>
+  </si>
+  <si>
+    <t>SILAS_SIMÕES</t>
+  </si>
+  <si>
+    <t>THIAGO_MONTEIRO</t>
+  </si>
+  <si>
+    <t>TIAGO_VIANA</t>
+  </si>
+  <si>
+    <t>VINICIUS_ROVARIS</t>
+  </si>
+  <si>
+    <t>WILLIAN_RODRIGUES</t>
+  </si>
+  <si>
+    <t>EDUARDO_VITAL</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>HUGO_DOS_SANTOS_GONÇALVES</t>
+  </si>
+  <si>
+    <t>RAUL_MARTINS_VENANCIO</t>
+  </si>
+  <si>
+    <t>RENAN_MIRANDA</t>
+  </si>
+  <si>
+    <t>SOFIA_KAZUE</t>
+  </si>
+  <si>
+    <t>YTALLO_GUEDES</t>
+  </si>
+  <si>
+    <t>MARIA_EDUARDA</t>
+  </si>
+  <si>
+    <t>AÇOS_VITAL</t>
+  </si>
+  <si>
+    <t>EUVERALDO_OLIVEIRA_DE_SOUZA</t>
+  </si>
+  <si>
+    <t>JOANES_OLIVEIRA</t>
+  </si>
+  <si>
+    <t>PRISCILA_YUMI_SAMEZIMA_MARC_DE_MOURA</t>
+  </si>
+  <si>
+    <t>WERESCLEY_DE_MOURA</t>
+  </si>
+  <si>
+    <t>JOAO_VITOR_MARTINS</t>
+  </si>
+  <si>
+    <t>LEONARDO_MARQUES_DIAS</t>
+  </si>
+  <si>
+    <t>Termo</t>
+  </si>
+  <si>
+    <t>ACOS VITAL</t>
+  </si>
+  <si>
+    <t>ANA_CAROLINE_VITAL</t>
+  </si>
+  <si>
+    <t>CARLOS_EDUARDO_BALATOR</t>
+  </si>
+  <si>
+    <t>MATEUS_ARAUJO</t>
+  </si>
+  <si>
+    <t>Ajuda de Custo</t>
+  </si>
+  <si>
+    <t>NÃO</t>
+  </si>
+  <si>
+    <t>0.35</t>
+  </si>
+  <si>
+    <t>0.1</t>
+  </si>
+  <si>
+    <t>PEDRO HENRIQUE</t>
+  </si>
+  <si>
+    <t>JOÃO VITOR</t>
+  </si>
+  <si>
+    <t>JOÃO PEDRO</t>
+  </si>
+  <si>
+    <t>SERGIO VITAL</t>
+  </si>
+  <si>
+    <t>EUVERALDO OLIVEIRA</t>
+  </si>
+  <si>
+    <t>ANTONIO PAIVA</t>
+  </si>
+  <si>
+    <t>CARLOS_HENRIQUE</t>
+  </si>
+  <si>
+    <t>DIEGO_FERNANDES</t>
+  </si>
+  <si>
+    <t>LUCAS_CACCIATORE</t>
+  </si>
+  <si>
+    <t>LEONARDO_MORAES</t>
+  </si>
+  <si>
+    <t>VINICIUS DINIZ</t>
+  </si>
+  <si>
     <t>DANIEL_SOUZA_DA_SILVA</t>
-  </si>
-  <si>
-    <t>DIEGO_JOSE_ARANTES</t>
-  </si>
-  <si>
-    <t>DIEGO_SOUSA_SANTOS</t>
-  </si>
-  <si>
-    <t>EBER_VIEIRA</t>
-  </si>
-  <si>
-    <t>EDCARLOS_SANTOS_DE_SOUZA</t>
-  </si>
-  <si>
-    <t>FLÁVIO_COUTINHO</t>
-  </si>
-  <si>
-    <t>GABRIEL_BARRETO</t>
-  </si>
-  <si>
-    <t>GABRIEL_DE_DEUS_NICOLAU</t>
-  </si>
-  <si>
-    <t>HUGO_FELIPE_DA_MATA</t>
-  </si>
-  <si>
-    <t>ISAQUE_CARVALHO_DO_ESPIRITO_SANTOS</t>
-  </si>
-  <si>
-    <t>JAMES_MADSON_OLIVEIRA_DE_SOUZA</t>
-  </si>
-  <si>
-    <t>JOARES_ALVES</t>
-  </si>
-  <si>
-    <t>JORGE_LUIZ</t>
-  </si>
-  <si>
-    <t>LARISSA_ALMEIDA</t>
-  </si>
-  <si>
-    <t>LEIDIANE_TEIXEIRA_COSTA</t>
-  </si>
-  <si>
-    <t>LEONARDO_APARECIDO_DE_MORAES</t>
-  </si>
-  <si>
-    <t>LEONARDO_PRATES</t>
-  </si>
-  <si>
-    <t>ROBERTA_SANTOS</t>
-  </si>
-  <si>
-    <t>RODRIGO_MIRANDA</t>
-  </si>
-  <si>
-    <t>RODRIGO_BERNARDINO</t>
-  </si>
-  <si>
-    <t>SARALIGIA_SIMÕES</t>
-  </si>
-  <si>
-    <t>SILAS_SIMÕES</t>
-  </si>
-  <si>
-    <t>THIAGO_MONTEIRO</t>
-  </si>
-  <si>
-    <t>TIAGO_VIANA</t>
-  </si>
-  <si>
-    <t>VINICIUS_ROVARIS</t>
-  </si>
-  <si>
-    <t>WILLIAN_RODRIGUES</t>
-  </si>
-  <si>
-    <t>EDUARDO_VITAL</t>
-  </si>
-  <si>
-    <t>MG</t>
-  </si>
-  <si>
-    <t>HUGO_DOS_SANTOS_GONÇALVES</t>
-  </si>
-  <si>
-    <t>RAUL_MARTINS_VENANCIO</t>
-  </si>
-  <si>
-    <t>RENAN_MIRANDA</t>
-  </si>
-  <si>
-    <t>SOFIA_KAZUE</t>
-  </si>
-  <si>
-    <t>YTALLO_GUEDES</t>
-  </si>
-  <si>
-    <t>MARIA_EDUARDA</t>
-  </si>
-  <si>
-    <t>AÇOS_VITAL</t>
-  </si>
-  <si>
-    <t>EUVERALDO_OLIVEIRA_DE_SOUZA</t>
-  </si>
-  <si>
-    <t>JOANES_OLIVEIRA</t>
-  </si>
-  <si>
-    <t>PRISCILA_YUMI_SAMEZIMA_MARC_DE_MOURA</t>
-  </si>
-  <si>
-    <t>WERESCLEY_DE_MOURA</t>
-  </si>
-  <si>
-    <t>JOAO_VITOR_MARTINS</t>
-  </si>
-  <si>
-    <t>LEONARDO_MARQUES_DIAS</t>
-  </si>
-  <si>
-    <t>Termo</t>
-  </si>
-  <si>
-    <t>ACOS VITAL</t>
-  </si>
-  <si>
-    <t>ANA_CAROLINE_VITAL</t>
-  </si>
-  <si>
-    <t>CARLOS_EDUARDO_BALATOR</t>
-  </si>
-  <si>
-    <t>MATEUS_ARAUJO</t>
-  </si>
-  <si>
-    <t>Ajuda de Custo</t>
-  </si>
-  <si>
-    <t>NÃO</t>
-  </si>
-  <si>
-    <t>0.35</t>
-  </si>
-  <si>
-    <t>0.1</t>
-  </si>
-  <si>
-    <t>PEDRO HENRIQUE</t>
-  </si>
-  <si>
-    <t>JOÃO VITOR</t>
-  </si>
-  <si>
-    <t>JOÃO PEDRO</t>
-  </si>
-  <si>
-    <t>SERGIO VITAL</t>
-  </si>
-  <si>
-    <t>EUVERALDO OLIVEIRA</t>
-  </si>
-  <si>
-    <t>ANTONIO PAIVA</t>
-  </si>
-  <si>
-    <t>CARLOS_HENRIQUE</t>
-  </si>
-  <si>
-    <t>DIEGO_FERNANDES</t>
-  </si>
-  <si>
-    <t>LUCAS_CACCIATORE</t>
   </si>
 </sst>
 </file>
@@ -649,7 +655,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -669,7 +675,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -688,13 +694,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D3" s="4">
         <v>5000</v>
@@ -708,7 +714,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D4" s="4">
         <v>0</v>
@@ -716,13 +722,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D5" s="4">
         <v>8000</v>
@@ -730,13 +736,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D6" s="4">
         <v>3500</v>
@@ -744,13 +750,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>7</v>
+        <v>63</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D7" s="4">
         <v>3500</v>
@@ -758,16 +764,16 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>64</v>
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D8" s="4">
-        <v>3500</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -778,10 +784,10 @@
         <v>4</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D9" s="4">
-        <v>12000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -792,10 +798,10 @@
         <v>4</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D10" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -809,12 +815,12 @@
         <v>5</v>
       </c>
       <c r="D11" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>4</v>
@@ -823,7 +829,7 @@
         <v>5</v>
       </c>
       <c r="D12" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -851,7 +857,7 @@
         <v>5</v>
       </c>
       <c r="D14" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -876,10 +882,10 @@
         <v>4</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="D16" s="4">
-        <v>0</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -890,10 +896,10 @@
         <v>4</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D17" s="4">
-        <v>20000</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -904,10 +910,10 @@
         <v>4</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="D18" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -918,7 +924,7 @@
         <v>4</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D19" s="4">
         <v>0</v>
@@ -935,7 +941,7 @@
         <v>5</v>
       </c>
       <c r="D20" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -953,28 +959,28 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="4">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
-        <v>65</v>
-      </c>
       <c r="B23" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D23" s="4">
         <v>0</v>
@@ -988,10 +994,10 @@
         <v>4</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D24" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -1002,7 +1008,7 @@
         <v>4</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D25" s="4">
         <v>3500</v>
@@ -1016,7 +1022,7 @@
         <v>4</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="D26" s="4">
         <v>3500</v>
@@ -1030,7 +1036,7 @@
         <v>4</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D27" s="4">
         <v>3500</v>
@@ -1058,10 +1064,10 @@
         <v>4</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="D29" s="4">
-        <v>3500</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
@@ -1072,10 +1078,10 @@
         <v>4</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D30" s="4">
-        <v>12000</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
@@ -1111,7 +1117,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>5</v>
@@ -1122,10 +1128,10 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>5</v>
@@ -1139,7 +1145,7 @@
         <v>35</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>5</v>
@@ -1153,7 +1159,7 @@
         <v>36</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>5</v>
@@ -1167,7 +1173,7 @@
         <v>37</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>5</v>
@@ -1181,7 +1187,7 @@
         <v>38</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>5</v>
@@ -1195,27 +1201,41 @@
         <v>39</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>5</v>
+        <v>53</v>
       </c>
       <c r="D39" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="D40" s="4">
-        <v>0</v>
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D41" s="4">
+        <v>3500</v>
       </c>
     </row>
   </sheetData>
@@ -1228,7 +1248,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -1241,42 +1261,42 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
@@ -1285,8 +1305,13 @@
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>12</v>
+      <c r="A11" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1304,12 +1329,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1339,18 +1364,18 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D2" s="2">
         <v>4500</v>
@@ -1358,13 +1383,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D3" s="2">
         <v>4500</v>
@@ -1372,13 +1397,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D4" s="2">
         <v>4500</v>
@@ -1386,13 +1411,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D5" s="2">
         <v>4500</v>
@@ -1400,13 +1425,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D6" s="2">
         <v>4500</v>
@@ -1414,13 +1439,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D7" s="2">
         <v>3500</v>

</xml_diff>

<commit_message>
ajuste para que o refaturamento seja considerado apenas o que estiver na planilha de bloqueios
</commit_message>
<xml_diff>
--- a/vendedores.xlsx
+++ b/vendedores.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TI\ROBERT\PROJETO COMISSOES\Script\extrator_comissoes_relatorio_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DCB7B3A-362E-4DC8-8318-77CFDBD5DF8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE36D99B-2C96-49DD-91BF-916EB27567D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VENDEDORES" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="71">
   <si>
     <t>Nome</t>
   </si>
@@ -96,154 +96,163 @@
     <t>JOARES_ALVES</t>
   </si>
   <si>
+    <t>LARISSA_ALMEIDA</t>
+  </si>
+  <si>
+    <t>LEIDIANE_TEIXEIRA_COSTA</t>
+  </si>
+  <si>
+    <t>LEONARDO_APARECIDO_DE_MORAES</t>
+  </si>
+  <si>
+    <t>LEONARDO_PRATES</t>
+  </si>
+  <si>
+    <t>ROBERTA_SANTOS</t>
+  </si>
+  <si>
+    <t>RODRIGO_MIRANDA</t>
+  </si>
+  <si>
+    <t>RODRIGO_BERNARDINO</t>
+  </si>
+  <si>
+    <t>SARALIGIA_SIMÕES</t>
+  </si>
+  <si>
+    <t>SILAS_SIMÕES</t>
+  </si>
+  <si>
+    <t>THIAGO_MONTEIRO</t>
+  </si>
+  <si>
+    <t>TIAGO_VIANA</t>
+  </si>
+  <si>
+    <t>VINICIUS_ROVARIS</t>
+  </si>
+  <si>
+    <t>WILLIAN_RODRIGUES</t>
+  </si>
+  <si>
+    <t>EDUARDO_VITAL</t>
+  </si>
+  <si>
+    <t>MG</t>
+  </si>
+  <si>
+    <t>HUGO_DOS_SANTOS_GONÇALVES</t>
+  </si>
+  <si>
+    <t>RAUL_MARTINS_VENANCIO</t>
+  </si>
+  <si>
+    <t>RENAN_MIRANDA</t>
+  </si>
+  <si>
+    <t>SOFIA_KAZUE</t>
+  </si>
+  <si>
+    <t>YTALLO_GUEDES</t>
+  </si>
+  <si>
+    <t>MARIA_EDUARDA</t>
+  </si>
+  <si>
+    <t>AÇOS_VITAL</t>
+  </si>
+  <si>
+    <t>EUVERALDO_OLIVEIRA_DE_SOUZA</t>
+  </si>
+  <si>
+    <t>JOANES_OLIVEIRA</t>
+  </si>
+  <si>
+    <t>PRISCILA_YUMI_SAMEZIMA_MARC_DE_MOURA</t>
+  </si>
+  <si>
+    <t>WERESCLEY_DE_MOURA</t>
+  </si>
+  <si>
+    <t>JOAO_VITOR_MARTINS</t>
+  </si>
+  <si>
+    <t>LEONARDO_MARQUES_DIAS</t>
+  </si>
+  <si>
+    <t>Termo</t>
+  </si>
+  <si>
+    <t>ACOS VITAL</t>
+  </si>
+  <si>
+    <t>ANA_CAROLINE_VITAL</t>
+  </si>
+  <si>
+    <t>CARLOS_EDUARDO_BALATOR</t>
+  </si>
+  <si>
+    <t>MATEUS_ARAUJO</t>
+  </si>
+  <si>
+    <t>Ajuda de Custo</t>
+  </si>
+  <si>
+    <t>NÃO</t>
+  </si>
+  <si>
+    <t>0.35</t>
+  </si>
+  <si>
+    <t>0.1</t>
+  </si>
+  <si>
+    <t>PEDRO HENRIQUE</t>
+  </si>
+  <si>
+    <t>JOÃO VITOR</t>
+  </si>
+  <si>
+    <t>JOÃO PEDRO</t>
+  </si>
+  <si>
+    <t>SERGIO VITAL</t>
+  </si>
+  <si>
+    <t>EUVERALDO OLIVEIRA</t>
+  </si>
+  <si>
+    <t>ANTONIO PAIVA</t>
+  </si>
+  <si>
+    <t>CARLOS_HENRIQUE</t>
+  </si>
+  <si>
+    <t>DIEGO_FERNANDES</t>
+  </si>
+  <si>
+    <t>LUCAS_CACCIATORE</t>
+  </si>
+  <si>
+    <t>LEONARDO_MORAES</t>
+  </si>
+  <si>
+    <t>DANIEL_SOUZA_DA_SILVA</t>
+  </si>
+  <si>
+    <t>PEDRO_HENRIQUE</t>
+  </si>
+  <si>
     <t>JORGE_LUIZ</t>
   </si>
   <si>
-    <t>LARISSA_ALMEIDA</t>
-  </si>
-  <si>
-    <t>LEIDIANE_TEIXEIRA_COSTA</t>
-  </si>
-  <si>
-    <t>LEONARDO_APARECIDO_DE_MORAES</t>
-  </si>
-  <si>
-    <t>LEONARDO_PRATES</t>
-  </si>
-  <si>
-    <t>ROBERTA_SANTOS</t>
-  </si>
-  <si>
-    <t>RODRIGO_MIRANDA</t>
-  </si>
-  <si>
-    <t>RODRIGO_BERNARDINO</t>
-  </si>
-  <si>
-    <t>SARALIGIA_SIMÕES</t>
-  </si>
-  <si>
-    <t>SILAS_SIMÕES</t>
-  </si>
-  <si>
-    <t>THIAGO_MONTEIRO</t>
-  </si>
-  <si>
-    <t>TIAGO_VIANA</t>
-  </si>
-  <si>
-    <t>VINICIUS_ROVARIS</t>
-  </si>
-  <si>
-    <t>WILLIAN_RODRIGUES</t>
-  </si>
-  <si>
-    <t>EDUARDO_VITAL</t>
-  </si>
-  <si>
-    <t>MG</t>
-  </si>
-  <si>
-    <t>HUGO_DOS_SANTOS_GONÇALVES</t>
-  </si>
-  <si>
-    <t>RAUL_MARTINS_VENANCIO</t>
-  </si>
-  <si>
-    <t>RENAN_MIRANDA</t>
-  </si>
-  <si>
-    <t>SOFIA_KAZUE</t>
-  </si>
-  <si>
-    <t>YTALLO_GUEDES</t>
-  </si>
-  <si>
-    <t>MARIA_EDUARDA</t>
-  </si>
-  <si>
-    <t>AÇOS_VITAL</t>
-  </si>
-  <si>
-    <t>EUVERALDO_OLIVEIRA_DE_SOUZA</t>
-  </si>
-  <si>
-    <t>JOANES_OLIVEIRA</t>
-  </si>
-  <si>
-    <t>PRISCILA_YUMI_SAMEZIMA_MARC_DE_MOURA</t>
-  </si>
-  <si>
-    <t>WERESCLEY_DE_MOURA</t>
-  </si>
-  <si>
-    <t>JOAO_VITOR_MARTINS</t>
-  </si>
-  <si>
-    <t>LEONARDO_MARQUES_DIAS</t>
-  </si>
-  <si>
-    <t>Termo</t>
-  </si>
-  <si>
-    <t>ACOS VITAL</t>
-  </si>
-  <si>
-    <t>ANA_CAROLINE_VITAL</t>
-  </si>
-  <si>
-    <t>CARLOS_EDUARDO_BALATOR</t>
-  </si>
-  <si>
-    <t>MATEUS_ARAUJO</t>
-  </si>
-  <si>
-    <t>Ajuda de Custo</t>
-  </si>
-  <si>
-    <t>NÃO</t>
-  </si>
-  <si>
-    <t>0.35</t>
-  </si>
-  <si>
-    <t>0.1</t>
-  </si>
-  <si>
-    <t>PEDRO HENRIQUE</t>
-  </si>
-  <si>
-    <t>JOÃO VITOR</t>
-  </si>
-  <si>
-    <t>JOÃO PEDRO</t>
-  </si>
-  <si>
-    <t>SERGIO VITAL</t>
-  </si>
-  <si>
-    <t>EUVERALDO OLIVEIRA</t>
-  </si>
-  <si>
-    <t>ANTONIO PAIVA</t>
-  </si>
-  <si>
-    <t>CARLOS_HENRIQUE</t>
-  </si>
-  <si>
-    <t>DIEGO_FERNANDES</t>
-  </si>
-  <si>
-    <t>LUCAS_CACCIATORE</t>
-  </si>
-  <si>
-    <t>LEONARDO_MORAES</t>
-  </si>
-  <si>
-    <t>VINICIUS DINIZ</t>
-  </si>
-  <si>
-    <t>DANIEL_SOUZA_DA_SILVA</t>
+    <t>DHIOVANNA_MACHADO</t>
+  </si>
+  <si>
+    <t>VINICIUS_DINIZ</t>
+  </si>
+  <si>
+    <t>KAROL_RODRIGUES</t>
   </si>
 </sst>
 </file>
@@ -655,7 +664,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -675,7 +684,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -694,13 +703,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D3" s="4">
         <v>5000</v>
@@ -714,7 +723,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D4" s="4">
         <v>0</v>
@@ -722,13 +731,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D5" s="4">
         <v>8000</v>
@@ -736,13 +745,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D6" s="4">
         <v>3500</v>
@@ -750,13 +759,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D7" s="4">
         <v>3500</v>
@@ -770,7 +779,7 @@
         <v>4</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D8" s="4">
         <v>12000</v>
@@ -784,7 +793,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D9" s="4">
         <v>0</v>
@@ -882,7 +891,7 @@
         <v>4</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D16" s="4">
         <v>20000</v>
@@ -910,7 +919,7 @@
         <v>4</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>53</v>
+        <v>5</v>
       </c>
       <c r="D18" s="4">
         <v>0</v>
@@ -927,7 +936,7 @@
         <v>5</v>
       </c>
       <c r="D19" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -945,28 +954,28 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D21" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D21" s="4">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
-        <v>64</v>
-      </c>
       <c r="B22" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D22" s="4">
         <v>0</v>
@@ -974,27 +983,27 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>53</v>
+        <v>5</v>
       </c>
       <c r="D23" s="4">
-        <v>0</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D24" s="4">
         <v>3500</v>
@@ -1002,7 +1011,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>4</v>
@@ -1016,13 +1025,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>53</v>
+        <v>5</v>
       </c>
       <c r="D26" s="4">
         <v>3500</v>
@@ -1030,7 +1039,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>4</v>
@@ -1044,7 +1053,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>4</v>
@@ -1058,21 +1067,21 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>53</v>
+        <v>5</v>
       </c>
       <c r="D29" s="4">
-        <v>12000</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>4</v>
@@ -1086,10 +1095,10 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>5</v>
@@ -1100,10 +1109,10 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>5</v>
@@ -1114,10 +1123,10 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>5</v>
@@ -1128,10 +1137,10 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>5</v>
@@ -1142,10 +1151,10 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>5</v>
@@ -1156,10 +1165,10 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>5</v>
@@ -1170,24 +1179,24 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="D37" s="4">
-        <v>3500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>38</v>
+        <v>64</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>5</v>
@@ -1198,44 +1207,30 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D39" s="4">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D40" s="4">
         <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D40" s="4">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D41" s="4">
-        <v>3500</v>
       </c>
     </row>
   </sheetData>
@@ -1248,7 +1243,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -1261,42 +1256,42 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
@@ -1311,7 +1306,27 @@
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1329,12 +1344,12 @@
   <sheetData>
     <row r="1" spans="1:1" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1364,18 +1379,18 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D2" s="2">
         <v>4500</v>
@@ -1383,13 +1398,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D3" s="2">
         <v>4500</v>
@@ -1397,13 +1412,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D4" s="2">
         <v>4500</v>
@@ -1411,13 +1426,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D5" s="2">
         <v>4500</v>
@@ -1425,13 +1440,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D6" s="2">
         <v>4500</v>
@@ -1439,13 +1454,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D7" s="2">
         <v>3500</v>

</xml_diff>

<commit_message>
Ajuste na busca retroativa, visando manter o status OK/ERRO
</commit_message>
<xml_diff>
--- a/vendedores.xlsx
+++ b/vendedores.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\TI\ROBERT\PROJETO COMISSOES\Script\extrator_comissoes_relatorio_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE36D99B-2C96-49DD-91BF-916EB27567D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56AD67B1-BC29-405E-BD1D-273CBE2A2E5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="71">
   <si>
     <t>Nome</t>
   </si>
@@ -664,7 +664,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -1233,6 +1233,20 @@
         <v>0</v>
       </c>
     </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D41" s="4">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1243,7 +1257,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -1321,11 +1335,6 @@
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>